<commit_message>
update & add tests
</commit_message>
<xml_diff>
--- a/excel_files/Testing.xlsx
+++ b/excel_files/Testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B05DE4-C419-47B3-B4AC-02571C92A606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19591A5E-AB2B-464C-8F10-CBDB10273D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{94B5C224-BB4D-4292-8301-349538C48A0E}"/>
+    <workbookView xWindow="-8220" yWindow="-13056" windowWidth="23232" windowHeight="12552" xr2:uid="{94B5C224-BB4D-4292-8301-349538C48A0E}"/>
   </bookViews>
   <sheets>
     <sheet name="AudioArt" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="167">
   <si>
     <t>package</t>
   </si>
@@ -517,13 +517,37 @@
   </si>
   <si>
     <t>test_convert_file</t>
+  </si>
+  <si>
+    <t>test_extract_walk_invalid_pattern</t>
+  </si>
+  <si>
+    <t>extract walk with invalid pattern</t>
+  </si>
+  <si>
+    <t>test_extract_walk_pattern</t>
+  </si>
+  <si>
+    <t>test_extract_walk</t>
+  </si>
+  <si>
+    <t>extract walk without a pattern</t>
+  </si>
+  <si>
+    <t>extract walk with a pattern</t>
+  </si>
+  <si>
+    <t>.m3u with testSetup built "PreppedMusic"</t>
+  </si>
+  <si>
+    <t>.mp3 w embedded in testSetup built "PreppedMusic"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -536,11 +560,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -640,7 +659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -649,9 +668,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1001,7 +1017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{240D0244-C07C-4B0D-B34B-DEFFB8A00779}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1062,7 +1078,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -1083,7 +1099,7 @@
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -1106,7 +1122,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1129,7 +1145,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -1138,7 +1154,7 @@
       <c r="C9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>55</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -1150,7 +1166,7 @@
       <c r="G9" s="3"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -1159,7 +1175,7 @@
       <c r="C10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>56</v>
       </c>
       <c r="E10" s="3" t="s">
@@ -1171,7 +1187,7 @@
       <c r="G10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1194,7 +1210,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -1217,7 +1233,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1240,7 +1256,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1261,7 +1277,7 @@
       <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -1282,7 +1298,7 @@
       <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1303,7 +1319,7 @@
       <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -1324,7 +1340,7 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="12" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1345,7 +1361,7 @@
       <c r="G18" s="3"/>
     </row>
     <row r="19" spans="1:7" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B19" s="5" t="s">
@@ -1354,86 +1370,132 @@
       <c r="C19" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="14" t="s">
+      <c r="D19" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F19" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="G19" s="14" t="s">
+      <c r="G19" s="13" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:7" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="G20" s="13"/>
+    </row>
+    <row r="21" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="G21" s="13"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="3" t="s">
+      <c r="B22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G20" s="3"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="G22" s="3"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D21" s="3" t="s">
+      <c r="B23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G21" s="3"/>
-    </row>
-    <row r="22" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="G23" s="3"/>
+    </row>
+    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D22" s="14" t="s">
+      <c r="B24" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F24" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="G22" s="15"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+      <c r="G24" s="14"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:G24">
-    <sortCondition ref="A6:A42"/>
-    <sortCondition ref="E6:E42"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:G26">
+    <sortCondition ref="A6:A44"/>
+    <sortCondition ref="E6:E44"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1502,7 +1564,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -1554,53 +1616,53 @@
       <c r="E9" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+    <row r="10" spans="1:7" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="16" t="s">
+      <c r="B10" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="15" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="16" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="16" t="s">
+    <row r="11" spans="1:7" s="15" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B11" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="15" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1625,10 +1687,10 @@
       <c r="A13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="19" t="s">
         <v>128</v>
       </c>
     </row>
@@ -1679,7 +1741,7 @@
       <c r="F19" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="19" t="s">
         <v>139</v>
       </c>
     </row>
@@ -1706,7 +1768,7 @@
       <c r="F22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="G22" s="21" t="s">
+      <c r="G22" s="20" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1714,7 +1776,7 @@
       <c r="F23" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G23" s="21"/>
+      <c r="G23" s="20"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">

</xml_diff>

<commit_message>
updates & add stub tests
</commit_message>
<xml_diff>
--- a/excel_files/Testing.xlsx
+++ b/excel_files/Testing.xlsx
@@ -1,26 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\excel_files\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{952C27F3-D7AB-4EDB-B8BE-BF6D56E5AED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="-8220" yWindow="-13056" windowWidth="23232" windowHeight="12552" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="AudioArt"/>
-    <sheet r:id="rId2" sheetId="2" name="AudioMetadata"/>
-    <sheet r:id="rId3" sheetId="3" name="AudioPlaylist"/>
-    <sheet r:id="rId4" sheetId="4" name="AudioNormalization"/>
-    <sheet r:id="rId5" sheetId="5" name="DirectoryProcessing"/>
-    <sheet r:id="rId6" sheetId="6" name="SubprocessUtilities"/>
-    <sheet r:id="rId7" sheetId="7" name="Main"/>
+    <sheet name="AudioArt" sheetId="1" r:id="rId1"/>
+    <sheet name="AudioMetadata" sheetId="2" r:id="rId2"/>
+    <sheet name="AudioPlaylist" sheetId="3" r:id="rId3"/>
+    <sheet name="AudioNormalization" sheetId="4" r:id="rId4"/>
+    <sheet name="DirectoryProcessing" sheetId="5" r:id="rId5"/>
+    <sheet name="SubprocessUtilities" sheetId="6" r:id="rId6"/>
+    <sheet name="Main" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="175">
   <si>
     <t>package</t>
   </si>
@@ -550,8 +556,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -573,7 +578,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -582,21 +587,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFbfbfbf"/>
+        <fgColor rgb="FFBFBFBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFdae3f3"/>
+        <fgColor rgb="FFDAE3F3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFe2f0d9"/>
+        <fgColor rgb="FFE2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -637,7 +648,7 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -646,7 +657,7 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
@@ -661,13 +672,13 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -676,13 +687,13 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -691,85 +702,143 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="30">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -780,10 +849,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -821,71 +890,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -913,7 +982,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -936,11 +1005,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -949,13 +1018,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -965,7 +1034,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -974,7 +1043,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -983,7 +1052,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -991,10 +1060,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1059,521 +1128,485 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="19.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="11.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="63.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="46.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="48.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="45.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="63" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="48.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="15" t="s">
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="6" t="s">
         <v>121</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="16" t="s">
+    <row r="9" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="B9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="G9" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="17" t="s">
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="B10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="G10" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="17" t="s">
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="B11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="6" t="s">
         <v>132</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="B12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="6" t="s">
         <v>136</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="18" t="s">
+    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="6" t="s">
         <v>140</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="14" t="s">
+    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="9" t="s">
+      <c r="B14" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="G14" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="16" t="s">
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" s="9" t="s">
+      <c r="B15" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G15" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="18" t="s">
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="B16" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="G16" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="14" t="s">
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="B17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="G17" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="15" t="s">
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="B18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G18" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="32.25">
-      <c r="A19" s="14" t="s">
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="B19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="9" t="s">
         <v>159</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="14" t="s">
+    <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="9" t="s">
+      <c r="B20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="G20" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="14" t="s">
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="B21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G21" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
-      <c r="A22" s="16" t="s">
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D22" s="9" t="s">
+      <c r="B22" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="G22" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="18" t="s">
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="B23" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G23" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="45.75">
-      <c r="A24" s="14" t="s">
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="12" t="s">
+      <c r="B24" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="F24" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="G24" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-      <c r="G26" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1581,737 +1614,768 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="23.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="22.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="32.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="47.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="118.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="23.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" customWidth="1"/>
+    <col min="5" max="5" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="118.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    </row>
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    </row>
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="5"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="7" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="9" t="s">
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="9" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="9" t="s">
+    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="45">
-      <c r="A9" s="8" t="s">
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="11" t="s">
+      <c r="B9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="45">
-      <c r="A10" s="8" t="s">
+    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="B10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="32.25">
-      <c r="A11" s="9" t="s">
+      <c r="G10" s="5"/>
+    </row>
+    <row r="11" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="12" t="s">
+      <c r="B11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="15" t="s">
         <v>43</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="45">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="12" t="s">
+      <c r="B12" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="16" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="33">
-      <c r="A14" s="8" t="s">
+      <c r="G13" s="21"/>
+    </row>
+    <row r="14" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="8" t="s">
+      <c r="B14" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="23" t="s">
         <v>55</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="16" t="s">
         <v>59</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="10" t="s">
+      <c r="B16" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="8" t="s">
+      <c r="G16" s="21"/>
+    </row>
+    <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8" t="s">
+      <c r="B17" s="22"/>
+      <c r="C17" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8" t="s">
+      <c r="E17" s="22"/>
+      <c r="F17" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="22" t="s">
         <v>65</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="10" t="s">
+    <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8" t="s">
+      <c r="E18" s="22"/>
+      <c r="F18" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="G18" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="32.25">
-      <c r="A19" s="8" t="s">
+      <c r="G18" s="22"/>
+    </row>
+    <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8" t="s">
+      <c r="B19" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8" t="s">
+      <c r="E19" s="24"/>
+      <c r="F19" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="25" t="s">
         <v>69</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="8" t="s">
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="9" t="s">
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22" t="s">
         <v>72</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="35.25">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2" t="s">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18">
-      <c r="A22" s="9" t="s">
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+    </row>
+    <row r="22" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2" t="s">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="8" t="s">
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+    </row>
+    <row r="23" spans="1:7" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8" t="s">
+      <c r="B23" s="27"/>
+      <c r="C23" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8" t="s">
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27" t="s">
         <v>74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18">
-      <c r="A24" s="5"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="10" t="s">
+    <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="9" t="s">
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
+    </row>
+    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="13" t="s">
+      <c r="B25" s="21"/>
+      <c r="C25" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="10"/>
-      <c r="F25" s="9" t="s">
+      <c r="E25" s="21"/>
+      <c r="F25" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="16" t="s">
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="9" t="s">
+    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="G26" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="8" t="s">
+      <c r="G26" s="16"/>
+    </row>
+    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8" t="s">
+      <c r="B27" s="22"/>
+      <c r="C27" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8" t="s">
+      <c r="E27" s="22"/>
+      <c r="F27" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="22" t="s">
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="10" t="s">
+    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8" t="s">
+      <c r="E28" s="22"/>
+      <c r="F28" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G28" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="9" t="s">
+      <c r="G28" s="22"/>
+    </row>
+    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="9" t="s">
+      <c r="B29" s="21"/>
+      <c r="C29" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="12" t="s">
+      <c r="G29" s="20" t="s">
         <v>86</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="9" t="s">
+    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="G30" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="9" t="s">
+      <c r="G30" s="21"/>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G31" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
-      <c r="A32" s="8" t="s">
+      <c r="G31" s="21"/>
+    </row>
+    <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="11" t="s">
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="23" t="s">
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
-      <c r="A33" s="9" t="s">
+    <row r="33" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="8" t="s">
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="E33" s="10"/>
-      <c r="F33" s="9" t="s">
+      <c r="E33" s="21"/>
+      <c r="F33" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="G33" s="16" t="s">
         <v>93</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10" t="s">
+    <row r="34" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="E34" s="10"/>
-      <c r="F34" s="9" t="s">
+      <c r="E34" s="21"/>
+      <c r="F34" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G34" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18">
-      <c r="A35" s="8" t="s">
+      <c r="G34" s="21"/>
+    </row>
+    <row r="35" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8" t="s">
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="G35" s="8" t="s">
+      <c r="G35" s="22" t="s">
         <v>97</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8" t="s">
+    <row r="36" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" s="22"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="G36" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8" t="s">
+      <c r="G36" s="22"/>
+    </row>
+    <row r="37" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B37" s="22"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="G37" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18">
-      <c r="A38" s="9" t="s">
+      <c r="G37" s="22"/>
+    </row>
+    <row r="38" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="9" t="s">
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="G38" s="16" t="s">
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="9" t="s">
+    <row r="39" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="G39" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18">
-      <c r="A40" s="8" t="s">
+      <c r="G39" s="21"/>
+    </row>
+    <row r="40" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8" t="s">
+      <c r="B40" s="22"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="G40" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8" t="s">
+      <c r="G40" s="22"/>
+    </row>
+    <row r="41" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="G41" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18">
-      <c r="A42" s="9" t="s">
+      <c r="G41" s="22"/>
+    </row>
+    <row r="42" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="9" t="s">
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="G42" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="9" t="s">
+      <c r="G42" s="21"/>
+    </row>
+    <row r="43" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18">
-      <c r="A44" s="8" t="s">
+      <c r="G43" s="21"/>
+    </row>
+    <row r="44" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8" t="s">
+      <c r="B44" s="22"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="G44" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8" t="s">
+      <c r="G44" s="22"/>
+    </row>
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="G45" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18">
-      <c r="A46" s="9" t="s">
+      <c r="G45" s="22"/>
+    </row>
+    <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18">
-      <c r="A47" s="8" t="s">
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
+    </row>
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18">
-      <c r="A48" s="9" t="s">
+      <c r="B47" s="22"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+    </row>
+    <row r="48" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="21"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2319,90 +2383,67 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="11.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="8.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="4.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="6.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2412,90 +2453,67 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="11.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="8.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="4.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="6.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2505,90 +2523,67 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="11.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="8.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="4.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="6.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2598,90 +2593,67 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="11.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="8.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="4.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="6.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2691,141 +2663,85 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="8.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="11.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="7.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="38.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="4.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="6.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    </row>
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2" t="s">
+    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
+    </row>
+    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+    </row>
+    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
+    </row>
+    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2" t="s">
+    </row>
+    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updates to metadata tests
</commit_message>
<xml_diff>
--- a/excel_files/Testing.xlsx
+++ b/excel_files/Testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{952C27F3-D7AB-4EDB-B8BE-BF6D56E5AED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3E51FF-A7FA-484A-81FB-0292DB2321DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8220" yWindow="-13056" windowWidth="23232" windowHeight="12552" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AudioArt" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="178">
   <si>
     <t>package</t>
   </si>
@@ -551,6 +551,15 @@
   </si>
   <si>
     <t>in tests/Music, 1 album dir w Folder.jpg, 1 album dir with jpg in AlbumArt, rest of album dirs w/o Folder.jpg</t>
+  </si>
+  <si>
+    <t>check if metadata_type = audio_file.__class__.__name__ is MP4</t>
+  </si>
+  <si>
+    <t>check if metadata_type = audio_file.__class__.__name__ is ASF</t>
+  </si>
+  <si>
+    <t>check if audio_file.__class__.__name__ is MP4/MP3/ASF</t>
   </si>
 </sst>
 </file>
@@ -744,7 +753,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -795,7 +804,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -811,12 +819,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -826,6 +828,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1781,13 +1786,13 @@
       <c r="C11" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>41</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="15" t="s">
@@ -1804,13 +1809,13 @@
       <c r="C12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="19" t="s">
         <v>44</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="20" t="s">
+      <c r="F12" s="19" t="s">
         <v>46</v>
       </c>
       <c r="G12" s="16" t="s">
@@ -1836,28 +1841,28 @@
       <c r="F13" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="21"/>
+      <c r="G13" s="20"/>
     </row>
     <row r="14" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="22" t="s">
+      <c r="B14" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="22" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1865,16 +1870,16 @@
       <c r="A15" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="21" t="s">
+      <c r="B15" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="D15" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="20" t="s">
         <v>57</v>
       </c>
       <c r="F15" s="16" t="s">
@@ -1888,92 +1893,92 @@
       <c r="A16" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="21" t="s">
+      <c r="B16" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="20" t="s">
         <v>61</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="21"/>
+      <c r="G16" s="20"/>
     </row>
     <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22" t="s">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22" t="s">
+      <c r="E17" s="21"/>
+      <c r="F17" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="21" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22" t="s">
+      <c r="B18" s="21"/>
+      <c r="C18" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22" t="s">
+      <c r="E18" s="21"/>
+      <c r="F18" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="G18" s="22"/>
+      <c r="G18" s="21"/>
     </row>
     <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="24" t="s">
+      <c r="B19" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24" t="s">
+      <c r="E19" s="16"/>
+      <c r="F19" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="19" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22" t="s">
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22" t="s">
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2007,50 +2012,50 @@
       <c r="F22" s="17"/>
       <c r="G22" s="17"/>
     </row>
-    <row r="23" spans="1:7" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="27" t="s">
+    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27" t="s">
+      <c r="B23" s="24"/>
+      <c r="C23" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="27" t="s">
+      <c r="D23" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27" t="s">
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="28" t="s">
+      <c r="B24" s="25"/>
+      <c r="C24" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="D24" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
     </row>
     <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21" t="s">
+      <c r="B25" s="20"/>
+      <c r="C25" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="21"/>
+      <c r="E25" s="20"/>
       <c r="F25" s="16" t="s">
         <v>77</v>
       </c>
@@ -2062,67 +2067,67 @@
       <c r="A26" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21" t="s">
+      <c r="B26" s="20"/>
+      <c r="C26" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
       <c r="F26" s="16" t="s">
         <v>79</v>
       </c>
       <c r="G26" s="16"/>
     </row>
     <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22" t="s">
+      <c r="B27" s="21"/>
+      <c r="C27" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="22" t="s">
+      <c r="D27" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22" t="s">
+      <c r="E27" s="21"/>
+      <c r="F27" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="G27" s="22" t="s">
+      <c r="G27" s="21" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22" t="s">
+      <c r="B28" s="21"/>
+      <c r="C28" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22" t="s">
+      <c r="E28" s="21"/>
+      <c r="F28" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="G28" s="22"/>
+      <c r="G28" s="21"/>
     </row>
     <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21" t="s">
+      <c r="B29" s="20"/>
+      <c r="C29" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="19" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2130,38 +2135,38 @@
       <c r="A30" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="G30" s="21"/>
+      <c r="G30" s="20"/>
     </row>
     <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
       <c r="F31" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G31" s="21"/>
+      <c r="G31" s="20"/>
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="23" t="s">
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="22" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2169,12 +2174,12 @@
       <c r="A33" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="21"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="24" t="s">
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="E33" s="21"/>
+      <c r="E33" s="20"/>
       <c r="F33" s="16" t="s">
         <v>92</v>
       </c>
@@ -2186,66 +2191,68 @@
       <c r="A34" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="21"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21" t="s">
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="E34" s="21"/>
+      <c r="E34" s="20"/>
       <c r="F34" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G34" s="21"/>
+      <c r="G34" s="20"/>
     </row>
     <row r="35" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22" t="s">
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="G35" s="22" t="s">
+      <c r="G35" s="21" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22" t="s">
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="G36" s="22"/>
+      <c r="G36" s="21"/>
     </row>
     <row r="37" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22" t="s">
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="G37" s="22"/>
-    </row>
-    <row r="38" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G37" s="21"/>
+    </row>
+    <row r="38" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="B38" s="21"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="27" t="s">
+        <v>177</v>
+      </c>
       <c r="F38" s="16" t="s">
         <v>77</v>
       </c>
@@ -2257,125 +2264,131 @@
       <c r="A39" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
       <c r="F39" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="G39" s="21"/>
-    </row>
-    <row r="40" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="22" t="s">
+      <c r="G39" s="20"/>
+    </row>
+    <row r="40" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22" t="s">
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="F40" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="G40" s="22"/>
+      <c r="G40" s="21"/>
     </row>
     <row r="41" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="22" t="s">
+      <c r="A41" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22" t="s">
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="G41" s="22"/>
-    </row>
-    <row r="42" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+    </row>
+    <row r="42" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="B42" s="21"/>
-      <c r="C42" s="21"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="27" t="s">
+        <v>175</v>
+      </c>
       <c r="F42" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="G42" s="21"/>
+      <c r="G42" s="20"/>
     </row>
     <row r="43" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="B43" s="21"/>
-      <c r="C43" s="21"/>
-      <c r="D43" s="21"/>
-      <c r="E43" s="21"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
       <c r="F43" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="21"/>
-    </row>
-    <row r="44" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="22" t="s">
+      <c r="G43" s="20"/>
+    </row>
+    <row r="44" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="B44" s="22"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22" t="s">
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="F44" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="G44" s="22"/>
+      <c r="G44" s="21"/>
     </row>
     <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22" t="s">
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="G45" s="22"/>
+      <c r="G45" s="21"/>
     </row>
     <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="B46" s="21"/>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
     </row>
     <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="22" t="s">
+      <c r="A47" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="B47" s="22"/>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
     </row>
     <row r="48" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="B48" s="21"/>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
removed not needed code in dir processing
</commit_message>
<xml_diff>
--- a/excel_files/Testing.xlsx
+++ b/excel_files/Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEABB477-7A55-4A99-8C0A-D1C5E1FB8F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1B0631-6963-478F-9640-53C0B222A073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="344">
   <si>
     <t>package</t>
   </si>
@@ -846,9 +846,6 @@
     <t>make_dir</t>
   </si>
   <si>
-    <t>move_audio_file</t>
-  </si>
-  <si>
     <t>path_info</t>
   </si>
   <si>
@@ -987,9 +984,6 @@
     <t>test_make_dir</t>
   </si>
   <si>
-    <t>fail path ExecError</t>
-  </si>
-  <si>
     <t>haqppy path</t>
   </si>
   <si>
@@ -1002,15 +996,9 @@
     <t>mock OSError?</t>
   </si>
   <si>
-    <t>test_move_audio_file</t>
-  </si>
-  <si>
     <t>test_remove_pattern</t>
   </si>
   <si>
-    <t>test_move_audio_file_fail</t>
-  </si>
-  <si>
     <t>test_remove_pattern_fail</t>
   </si>
   <si>
@@ -1051,12 +1039,6 @@
   </si>
   <si>
     <t>mock OSError with errno == EACCES?</t>
-  </si>
-  <si>
-    <t>a file from /tests/Music</t>
-  </si>
-  <si>
-    <t>non-extant file? Mock ExecError?</t>
   </si>
   <si>
     <t>create temp /tests/tld/artist/album</t>
@@ -3677,7 +3659,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" style="42" bestFit="1" customWidth="1"/>
@@ -3773,16 +3755,16 @@
         <v>19</v>
       </c>
       <c r="D7" s="41" t="s">
+        <v>295</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>294</v>
+      </c>
+      <c r="F7" s="41" t="s">
         <v>296</v>
       </c>
-      <c r="E7" s="42" t="s">
-        <v>295</v>
-      </c>
-      <c r="F7" s="41" t="s">
-        <v>297</v>
-      </c>
       <c r="G7" s="41" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -3796,16 +3778,16 @@
         <v>19</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E8" s="45" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F8" s="45" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G8" s="46" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3819,13 +3801,13 @@
         <v>19</v>
       </c>
       <c r="D9" s="47" t="s">
+        <v>302</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>301</v>
+      </c>
+      <c r="F9" s="47" t="s">
         <v>303</v>
-      </c>
-      <c r="E9" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="F9" s="47" t="s">
-        <v>304</v>
       </c>
       <c r="G9" s="47"/>
     </row>
@@ -3840,13 +3822,13 @@
         <v>19</v>
       </c>
       <c r="D10" s="45" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E10" s="45" t="s">
+        <v>304</v>
+      </c>
+      <c r="F10" s="45" t="s">
         <v>305</v>
-      </c>
-      <c r="F10" s="45" t="s">
-        <v>306</v>
       </c>
       <c r="G10" s="45"/>
     </row>
@@ -3861,13 +3843,13 @@
         <v>19</v>
       </c>
       <c r="D11" s="45" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F11" s="45" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G11" s="45"/>
     </row>
@@ -3882,13 +3864,13 @@
         <v>19</v>
       </c>
       <c r="D12" s="45" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E12" s="45" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F12" s="45" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G12" s="45"/>
     </row>
@@ -3903,13 +3885,13 @@
         <v>19</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E13" s="45" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F13" s="45" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G13" s="45"/>
     </row>
@@ -3966,16 +3948,16 @@
         <v>19</v>
       </c>
       <c r="D16" s="49" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E16" s="49" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F16" s="49" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="G16" s="49" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="52" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3989,16 +3971,16 @@
         <v>207</v>
       </c>
       <c r="D17" s="49" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="E17" s="49" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="F17" s="49" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="G17" s="49" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="52" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4012,19 +3994,19 @@
         <v>207</v>
       </c>
       <c r="D18" s="49" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E18" s="49" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="F18" s="49" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="G18" s="49" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" s="52" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="50" t="s">
         <v>271</v>
       </c>
@@ -4032,22 +4014,20 @@
         <v>19</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>207</v>
+        <v>19</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>100</v>
+        <v>272</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>323</v>
+        <v>273</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>340</v>
-      </c>
-      <c r="G19" s="51" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" s="52" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>274</v>
+      </c>
+      <c r="G19" s="51"/>
+    </row>
+    <row r="20" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="50" t="s">
         <v>271</v>
       </c>
@@ -4055,84 +4035,86 @@
         <v>19</v>
       </c>
       <c r="C20" s="51" t="s">
-        <v>207</v>
+        <v>19</v>
       </c>
       <c r="D20" s="51" t="s">
-        <v>318</v>
+        <v>275</v>
       </c>
       <c r="E20" s="51" t="s">
-        <v>325</v>
+        <v>276</v>
       </c>
       <c r="F20" s="51" t="s">
-        <v>341</v>
-      </c>
-      <c r="G20" s="51" t="s">
-        <v>347</v>
-      </c>
+        <v>277</v>
+      </c>
+      <c r="G20" s="51"/>
     </row>
     <row r="21" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="48" t="s">
-        <v>272</v>
-      </c>
-      <c r="B21" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="49" t="s">
-        <v>273</v>
-      </c>
-      <c r="E21" s="49" t="s">
-        <v>274</v>
-      </c>
-      <c r="F21" s="49" t="s">
-        <v>275</v>
-      </c>
-      <c r="G21" s="49"/>
+        <v>278</v>
+      </c>
+      <c r="B21" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="D21" s="48" t="s">
+        <v>317</v>
+      </c>
+      <c r="E21" s="48" t="s">
+        <v>324</v>
+      </c>
+      <c r="F21" s="48" t="s">
+        <v>336</v>
+      </c>
+      <c r="G21" s="48" t="s">
+        <v>337</v>
+      </c>
     </row>
     <row r="22" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="48" t="s">
-        <v>272</v>
-      </c>
-      <c r="B22" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="D22" s="49" t="s">
-        <v>276</v>
-      </c>
-      <c r="E22" s="49" t="s">
-        <v>277</v>
-      </c>
-      <c r="F22" s="49" t="s">
         <v>278</v>
       </c>
-      <c r="G22" s="49"/>
+      <c r="B22" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="D22" s="48" t="s">
+        <v>330</v>
+      </c>
+      <c r="E22" s="48" t="s">
+        <v>332</v>
+      </c>
+      <c r="F22" s="48" t="s">
+        <v>338</v>
+      </c>
+      <c r="G22" s="48" t="s">
+        <v>337</v>
+      </c>
     </row>
     <row r="23" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="s">
-        <v>279</v>
-      </c>
-      <c r="B23" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="C23" s="51" t="s">
+      <c r="A23" s="48" t="s">
+        <v>278</v>
+      </c>
+      <c r="B23" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="48" t="s">
         <v>207</v>
       </c>
-      <c r="D23" s="51" t="s">
-        <v>319</v>
-      </c>
-      <c r="E23" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="F23" s="51" t="s">
-        <v>342</v>
-      </c>
-      <c r="G23" s="51" t="s">
-        <v>343</v>
+      <c r="D23" s="48" t="s">
+        <v>331</v>
+      </c>
+      <c r="E23" s="48" t="s">
+        <v>323</v>
+      </c>
+      <c r="F23" s="48" t="s">
+        <v>335</v>
+      </c>
+      <c r="G23" s="48" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="24" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -4146,16 +4128,16 @@
         <v>207</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>334</v>
+        <v>100</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
       <c r="F24" s="51" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="G24" s="51" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -4169,85 +4151,39 @@
         <v>207</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="F25" s="51" t="s">
         <v>339</v>
       </c>
       <c r="G25" s="51" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="48" t="s">
-        <v>280</v>
-      </c>
-      <c r="B26" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26" s="49" t="s">
+      <c r="A26" s="50" t="s">
+        <v>279</v>
+      </c>
+      <c r="B26" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="D26" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="E26" s="49" t="s">
-        <v>324</v>
-      </c>
-      <c r="F26" s="49" t="s">
-        <v>348</v>
-      </c>
-      <c r="G26" s="49" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="48" t="s">
-        <v>280</v>
-      </c>
-      <c r="B27" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="49" t="s">
-        <v>207</v>
-      </c>
-      <c r="D27" s="49" t="s">
-        <v>337</v>
-      </c>
-      <c r="E27" s="49" t="s">
-        <v>326</v>
-      </c>
-      <c r="F27" s="49" t="s">
-        <v>345</v>
-      </c>
-      <c r="G27" s="49" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" s="52" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="48" t="s">
-        <v>280</v>
-      </c>
-      <c r="B28" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="49" t="s">
-        <v>207</v>
-      </c>
-      <c r="D28" s="49" t="s">
-        <v>338</v>
-      </c>
-      <c r="E28" s="49" t="s">
-        <v>329</v>
-      </c>
-      <c r="F28" s="49" t="s">
-        <v>339</v>
-      </c>
-      <c r="G28" s="49" t="s">
-        <v>339</v>
+      <c r="D26" s="51" t="s">
+        <v>334</v>
+      </c>
+      <c r="E26" s="51" t="s">
+        <v>325</v>
+      </c>
+      <c r="F26" s="51" t="s">
+        <v>335</v>
+      </c>
+      <c r="G26" s="51" t="s">
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4275,7 +4211,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4283,7 +4219,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4333,7 +4269,7 @@
     </row>
     <row r="6" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>19</v>
@@ -4345,18 +4281,18 @@
         <v>108</v>
       </c>
       <c r="E6" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="G6" s="14" t="s">
         <v>285</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>19</v>
@@ -4368,13 +4304,13 @@
         <v>108</v>
       </c>
       <c r="E7" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="G7" s="12" t="s">
         <v>288</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>285</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -4436,7 +4372,7 @@
       <c r="B5" s="39"/>
       <c r="C5" s="39"/>
       <c r="D5" s="39" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E5" s="39"/>
       <c r="F5" s="39"/>
@@ -4447,7 +4383,7 @@
       <c r="B6" s="39"/>
       <c r="C6" s="39"/>
       <c r="D6" s="39" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E6" s="39"/>
       <c r="F6" s="39"/>
@@ -4458,7 +4394,7 @@
       <c r="B7" s="39"/>
       <c r="C7" s="39"/>
       <c r="D7" s="39" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E7" s="39"/>
       <c r="F7" s="39"/>
@@ -4469,7 +4405,7 @@
       <c r="B8" s="39"/>
       <c r="C8" s="39"/>
       <c r="D8" s="39" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E8" s="39"/>
       <c r="F8" s="39"/>
@@ -4480,7 +4416,7 @@
       <c r="B9" s="39"/>
       <c r="C9" s="39"/>
       <c r="D9" s="39" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E9" s="39"/>
       <c r="F9" s="39"/>

</xml_diff>